<commit_message>
Fix all critical template bugs and add Gumroad assets
- Fix broken P&L formula (IF/OR nested incorrectly) in Trade Log
- Fix all Trade Log formulas for 50 trade entries (rows 5-54)
- Fix Dashboard formulas: win rate, avg win/loss, profit factor, worst trade
- Fix Analytics: remove Cumulative P&L vs Monthly section overlap
- Fix December invalid date (2026-13-01 -> 2027-01-01)
- Fix Analytics monthly Win Rate and Avg R formulas row references
- Extend Cumulative P&L section to 10 trades
- Add thumbnail.png (1280x720) for Gumroad cover image
- Update GUMROAD_LISTING.md claims to match reality
- Recreate Delivery_Instructions.pdf with correct template link
</commit_message>
<xml_diff>
--- a/Pro_Trading_Journal_Template.xlsx
+++ b/Pro_Trading_Journal_Template.xlsx
@@ -19,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +77,10 @@
       <color rgb="001B2A4A"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -95,7 +100,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -122,11 +127,26 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="001B2A4A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="001B2A4A"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,6 +212,40 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -559,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:T54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -585,11 +639,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>PRO TRADING JOURNAL</t>
         </is>
       </c>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -749,20 +806,24 @@
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="M5" s="7" t="n">
-        <v>770</v>
-      </c>
-      <c r="N5" s="8" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="O5" s="9" t="n">
-        <v>2.2</v>
+      <c r="M5" s="39">
+        <f>IF(OR(E5="",K5=""),"",IF(E5="Long",(K5-G5)*J5,IF(E5="Short",(G5-K5)*J5,"")))</f>
+        <v/>
+      </c>
+      <c r="N5" s="8">
+        <f>IF(OR(E5="",K5="",G5=0),"",IF(E5="Long",(K5-G5)/G5,IF(E5="Short",(G5-K5)/G5,"")))</f>
+        <v/>
+      </c>
+      <c r="O5" s="9">
+        <f>IF(OR(M5="",H5=""),"",IF(ABS(J5*(G5-H5))=0,"N/A",M5/ABS(J5*(G5-H5))))</f>
+        <v/>
       </c>
       <c r="P5" s="6" t="n">
         <v>1.5</v>
       </c>
-      <c r="Q5" s="7" t="n">
-        <v>768.5</v>
+      <c r="Q5" s="39">
+        <f>IF(M5="","",M5-P5)</f>
+        <v/>
       </c>
       <c r="R5" s="4" t="inlineStr">
         <is>
@@ -824,20 +885,24 @@
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="M6" s="13" t="n">
-        <v>-800</v>
-      </c>
-      <c r="N6" s="14" t="n">
-        <v>-0.0078</v>
-      </c>
-      <c r="O6" s="15" t="n">
-        <v>-0.57</v>
+      <c r="M6" s="40">
+        <f>IF(OR(E6="",K6=""),"",IF(E6="Long",(K6-G6)*J6,IF(E6="Short",(G6-K6)*J6,"")))</f>
+        <v/>
+      </c>
+      <c r="N6" s="14">
+        <f>IF(OR(E6="",K6="",G6=0),"",IF(E6="Long",(K6-G6)/G6,IF(E6="Short",(G6-K6)/G6,"")))</f>
+        <v/>
+      </c>
+      <c r="O6" s="15">
+        <f>IF(OR(M6="",H6=""),"",IF(ABS(J6*(G6-H6))=0,"N/A",M6/ABS(J6*(G6-H6))))</f>
+        <v/>
       </c>
       <c r="P6" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="Q6" s="13" t="n">
-        <v>-803</v>
+      <c r="Q6" s="40">
+        <f>IF(M6="","",M6-P6)</f>
+        <v/>
       </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
@@ -900,20 +965,24 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="M7" s="7" t="n">
-        <v>675</v>
-      </c>
-      <c r="N7" s="8" t="n">
-        <v>0.0433</v>
-      </c>
-      <c r="O7" s="9" t="n">
-        <v>2.25</v>
+      <c r="M7" s="39">
+        <f>IF(OR(E7="",K7=""),"",IF(E7="Long",(K7-G7)*J7,IF(E7="Short",(G7-K7)*J7,"")))</f>
+        <v/>
+      </c>
+      <c r="N7" s="8">
+        <f>IF(OR(E7="",K7="",G7=0),"",IF(E7="Long",(K7-G7)/G7,IF(E7="Short",(G7-K7)/G7,"")))</f>
+        <v/>
+      </c>
+      <c r="O7" s="9">
+        <f>IF(OR(M7="",H7=""),"",IF(ABS(J7*(G7-H7))=0,"N/A",M7/ABS(J7*(G7-H7))))</f>
+        <v/>
       </c>
       <c r="P7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="Q7" s="7" t="n">
-        <v>674</v>
+      <c r="Q7" s="39">
+        <f>IF(M7="","",M7-P7)</f>
+        <v/>
       </c>
       <c r="R7" s="4" t="inlineStr"/>
       <c r="S7" s="4" t="inlineStr">
@@ -971,20 +1040,24 @@
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="M8" s="17" t="n">
-        <v>30</v>
-      </c>
-      <c r="N8" s="18" t="n">
-        <v>0.0091</v>
-      </c>
-      <c r="O8" s="15" t="n">
-        <v>1.5</v>
+      <c r="M8" s="41">
+        <f>IF(OR(E8="",K8=""),"",IF(E8="Long",(K8-G8)*J8,IF(E8="Short",(G8-K8)*J8,"")))</f>
+        <v/>
+      </c>
+      <c r="N8" s="18">
+        <f>IF(OR(E8="",K8="",G8=0),"",IF(E8="Long",(K8-G8)/G8,IF(E8="Short",(G8-K8)/G8,"")))</f>
+        <v/>
+      </c>
+      <c r="O8" s="15">
+        <f>IF(OR(M8="",H8=""),"",IF(ABS(J8*(G8-H8))=0,"N/A",M8/ABS(J8*(G8-H8))))</f>
+        <v/>
       </c>
       <c r="P8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="Q8" s="17" t="n">
-        <v>28</v>
+      <c r="Q8" s="41">
+        <f>IF(M8="","",M8-P8)</f>
+        <v/>
       </c>
       <c r="R8" s="10" t="inlineStr"/>
       <c r="S8" s="10" t="inlineStr">
@@ -1037,13 +1110,25 @@
       </c>
       <c r="K9" s="6" t="n"/>
       <c r="L9" s="4" t="n"/>
-      <c r="M9" s="4" t="n"/>
-      <c r="N9" s="4" t="n"/>
-      <c r="O9" s="4" t="n"/>
+      <c r="M9" s="42">
+        <f>IF(OR(E9="",K9=""),"",IF(E9="Long",(K9-G9)*J9,IF(E9="Short",(G9-K9)*J9,"")))</f>
+        <v/>
+      </c>
+      <c r="N9" s="34">
+        <f>IF(OR(E9="",K9="",G9=0),"",IF(E9="Long",(K9-G9)/G9,IF(E9="Short",(G9-K9)/G9,"")))</f>
+        <v/>
+      </c>
+      <c r="O9" s="4">
+        <f>IF(OR(M9="",H9=""),"",IF(ABS(J9*(G9-H9))=0,"N/A",M9/ABS(J9*(G9-H9))))</f>
+        <v/>
+      </c>
       <c r="P9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="Q9" s="4" t="n"/>
+      <c r="Q9" s="42">
+        <f>IF(M9="","",M9-P9)</f>
+        <v/>
+      </c>
       <c r="R9" s="4" t="inlineStr"/>
       <c r="S9" s="4" t="inlineStr">
         <is>
@@ -1052,254 +1137,947 @@
       </c>
     </row>
     <row r="10">
-      <c r="M10">
-        <f>IF(OR(K10="",(E10="Long")*(K10-G10)*J10,(E10="Short")*(G10-K10)*J10))</f>
-        <v/>
-      </c>
-      <c r="N10">
-        <f>IF(G10=0,"",M10/(G10*J10))</f>
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="43">
+        <f>IF(OR(E10="",K10=""),"",IF(E10="Long",(K10-G10)*J10,IF(E10="Short",(G10-K10)*J10,"")))</f>
+        <v/>
+      </c>
+      <c r="N10" s="44">
+        <f>IF(OR(E10="",K10="",G10=0),"",IF(E10="Long",(K10-G10)/G10,IF(E10="Short",(G10-K10)/G10,"")))</f>
         <v/>
       </c>
       <c r="O10">
-        <f>IF(OR(G10=H10,J10=0),"",M10/(ABS(G10-H10)*J10))</f>
-        <v/>
-      </c>
-      <c r="Q10">
+        <f>IF(OR(M10="",H10=""),"",IF(ABS(J10*(G10-H10))=0,"N/A",M10/ABS(J10*(G10-H10))))</f>
+        <v/>
+      </c>
+      <c r="Q10" s="43">
         <f>IF(M10="","",M10-P10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="M11">
-        <f>IF(OR(K11="",(E11="Long")*(K11-G11)*J11,(E11="Short")*(G11-K11)*J11))</f>
-        <v/>
-      </c>
-      <c r="N11">
-        <f>IF(G11=0,"",M11/(G11*J11))</f>
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" s="43">
+        <f>IF(OR(E11="",K11=""),"",IF(E11="Long",(K11-G11)*J11,IF(E11="Short",(G11-K11)*J11,"")))</f>
+        <v/>
+      </c>
+      <c r="N11" s="44">
+        <f>IF(OR(E11="",K11="",G11=0),"",IF(E11="Long",(K11-G11)/G11,IF(E11="Short",(G11-K11)/G11,"")))</f>
         <v/>
       </c>
       <c r="O11">
-        <f>IF(OR(G11=H11,J11=0),"",M11/(ABS(G11-H11)*J11))</f>
-        <v/>
-      </c>
-      <c r="Q11">
+        <f>IF(OR(M11="",H11=""),"",IF(ABS(J11*(G11-H11))=0,"N/A",M11/ABS(J11*(G11-H11))))</f>
+        <v/>
+      </c>
+      <c r="Q11" s="43">
         <f>IF(M11="","",M11-P11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="M12">
-        <f>IF(OR(K12="",(E12="Long")*(K12-G12)*J12,(E12="Short")*(G12-K12)*J12))</f>
-        <v/>
-      </c>
-      <c r="N12">
-        <f>IF(G12=0,"",M12/(G12*J12))</f>
+      <c r="A12" t="n">
+        <v>8</v>
+      </c>
+      <c r="M12" s="43">
+        <f>IF(OR(E12="",K12=""),"",IF(E12="Long",(K12-G12)*J12,IF(E12="Short",(G12-K12)*J12,"")))</f>
+        <v/>
+      </c>
+      <c r="N12" s="44">
+        <f>IF(OR(E12="",K12="",G12=0),"",IF(E12="Long",(K12-G12)/G12,IF(E12="Short",(G12-K12)/G12,"")))</f>
         <v/>
       </c>
       <c r="O12">
-        <f>IF(OR(G12=H12,J12=0),"",M12/(ABS(G12-H12)*J12))</f>
-        <v/>
-      </c>
-      <c r="Q12">
+        <f>IF(OR(M12="",H12=""),"",IF(ABS(J12*(G12-H12))=0,"N/A",M12/ABS(J12*(G12-H12))))</f>
+        <v/>
+      </c>
+      <c r="Q12" s="43">
         <f>IF(M12="","",M12-P12)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="M13">
-        <f>IF(OR(K13="",(E13="Long")*(K13-G13)*J13,(E13="Short")*(G13-K13)*J13))</f>
-        <v/>
-      </c>
-      <c r="N13">
-        <f>IF(G13=0,"",M13/(G13*J13))</f>
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="M13" s="43">
+        <f>IF(OR(E13="",K13=""),"",IF(E13="Long",(K13-G13)*J13,IF(E13="Short",(G13-K13)*J13,"")))</f>
+        <v/>
+      </c>
+      <c r="N13" s="44">
+        <f>IF(OR(E13="",K13="",G13=0),"",IF(E13="Long",(K13-G13)/G13,IF(E13="Short",(G13-K13)/G13,"")))</f>
         <v/>
       </c>
       <c r="O13">
-        <f>IF(OR(G13=H13,J13=0),"",M13/(ABS(G13-H13)*J13))</f>
-        <v/>
-      </c>
-      <c r="Q13">
+        <f>IF(OR(M13="",H13=""),"",IF(ABS(J13*(G13-H13))=0,"N/A",M13/ABS(J13*(G13-H13))))</f>
+        <v/>
+      </c>
+      <c r="Q13" s="43">
         <f>IF(M13="","",M13-P13)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="M14">
-        <f>IF(OR(K14="",(E14="Long")*(K14-G14)*J14,(E14="Short")*(G14-K14)*J14))</f>
-        <v/>
-      </c>
-      <c r="N14">
-        <f>IF(G14=0,"",M14/(G14*J14))</f>
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="M14" s="43">
+        <f>IF(OR(E14="",K14=""),"",IF(E14="Long",(K14-G14)*J14,IF(E14="Short",(G14-K14)*J14,"")))</f>
+        <v/>
+      </c>
+      <c r="N14" s="44">
+        <f>IF(OR(E14="",K14="",G14=0),"",IF(E14="Long",(K14-G14)/G14,IF(E14="Short",(G14-K14)/G14,"")))</f>
         <v/>
       </c>
       <c r="O14">
-        <f>IF(OR(G14=H14,J14=0),"",M14/(ABS(G14-H14)*J14))</f>
-        <v/>
-      </c>
-      <c r="Q14">
+        <f>IF(OR(M14="",H14=""),"",IF(ABS(J14*(G14-H14))=0,"N/A",M14/ABS(J14*(G14-H14))))</f>
+        <v/>
+      </c>
+      <c r="Q14" s="43">
         <f>IF(M14="","",M14-P14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="M15">
-        <f>IF(OR(K15="",(E15="Long")*(K15-G15)*J15,(E15="Short")*(G15-K15)*J15))</f>
-        <v/>
-      </c>
-      <c r="N15">
-        <f>IF(G15=0,"",M15/(G15*J15))</f>
+      <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="M15" s="43">
+        <f>IF(OR(E15="",K15=""),"",IF(E15="Long",(K15-G15)*J15,IF(E15="Short",(G15-K15)*J15,"")))</f>
+        <v/>
+      </c>
+      <c r="N15" s="44">
+        <f>IF(OR(E15="",K15="",G15=0),"",IF(E15="Long",(K15-G15)/G15,IF(E15="Short",(G15-K15)/G15,"")))</f>
         <v/>
       </c>
       <c r="O15">
-        <f>IF(OR(G15=H15,J15=0),"",M15/(ABS(G15-H15)*J15))</f>
-        <v/>
-      </c>
-      <c r="Q15">
+        <f>IF(OR(M15="",H15=""),"",IF(ABS(J15*(G15-H15))=0,"N/A",M15/ABS(J15*(G15-H15))))</f>
+        <v/>
+      </c>
+      <c r="Q15" s="43">
         <f>IF(M15="","",M15-P15)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="M16">
-        <f>IF(OR(K16="",(E16="Long")*(K16-G16)*J16,(E16="Short")*(G16-K16)*J16))</f>
-        <v/>
-      </c>
-      <c r="N16">
-        <f>IF(G16=0,"",M16/(G16*J16))</f>
+      <c r="A16" t="n">
+        <v>12</v>
+      </c>
+      <c r="M16" s="43">
+        <f>IF(OR(E16="",K16=""),"",IF(E16="Long",(K16-G16)*J16,IF(E16="Short",(G16-K16)*J16,"")))</f>
+        <v/>
+      </c>
+      <c r="N16" s="44">
+        <f>IF(OR(E16="",K16="",G16=0),"",IF(E16="Long",(K16-G16)/G16,IF(E16="Short",(G16-K16)/G16,"")))</f>
         <v/>
       </c>
       <c r="O16">
-        <f>IF(OR(G16=H16,J16=0),"",M16/(ABS(G16-H16)*J16))</f>
-        <v/>
-      </c>
-      <c r="Q16">
+        <f>IF(OR(M16="",H16=""),"",IF(ABS(J16*(G16-H16))=0,"N/A",M16/ABS(J16*(G16-H16))))</f>
+        <v/>
+      </c>
+      <c r="Q16" s="43">
         <f>IF(M16="","",M16-P16)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="M17">
-        <f>IF(OR(K17="",(E17="Long")*(K17-G17)*J17,(E17="Short")*(G17-K17)*J17))</f>
-        <v/>
-      </c>
-      <c r="N17">
-        <f>IF(G17=0,"",M17/(G17*J17))</f>
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="M17" s="43">
+        <f>IF(OR(E17="",K17=""),"",IF(E17="Long",(K17-G17)*J17,IF(E17="Short",(G17-K17)*J17,"")))</f>
+        <v/>
+      </c>
+      <c r="N17" s="44">
+        <f>IF(OR(E17="",K17="",G17=0),"",IF(E17="Long",(K17-G17)/G17,IF(E17="Short",(G17-K17)/G17,"")))</f>
         <v/>
       </c>
       <c r="O17">
-        <f>IF(OR(G17=H17,J17=0),"",M17/(ABS(G17-H17)*J17))</f>
-        <v/>
-      </c>
-      <c r="Q17">
+        <f>IF(OR(M17="",H17=""),"",IF(ABS(J17*(G17-H17))=0,"N/A",M17/ABS(J17*(G17-H17))))</f>
+        <v/>
+      </c>
+      <c r="Q17" s="43">
         <f>IF(M17="","",M17-P17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="M18">
-        <f>IF(OR(K18="",(E18="Long")*(K18-G18)*J18,(E18="Short")*(G18-K18)*J18))</f>
-        <v/>
-      </c>
-      <c r="N18">
-        <f>IF(G18=0,"",M18/(G18*J18))</f>
+      <c r="A18" t="n">
+        <v>14</v>
+      </c>
+      <c r="M18" s="43">
+        <f>IF(OR(E18="",K18=""),"",IF(E18="Long",(K18-G18)*J18,IF(E18="Short",(G18-K18)*J18,"")))</f>
+        <v/>
+      </c>
+      <c r="N18" s="44">
+        <f>IF(OR(E18="",K18="",G18=0),"",IF(E18="Long",(K18-G18)/G18,IF(E18="Short",(G18-K18)/G18,"")))</f>
         <v/>
       </c>
       <c r="O18">
-        <f>IF(OR(G18=H18,J18=0),"",M18/(ABS(G18-H18)*J18))</f>
-        <v/>
-      </c>
-      <c r="Q18">
+        <f>IF(OR(M18="",H18=""),"",IF(ABS(J18*(G18-H18))=0,"N/A",M18/ABS(J18*(G18-H18))))</f>
+        <v/>
+      </c>
+      <c r="Q18" s="43">
         <f>IF(M18="","",M18-P18)</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="M19">
-        <f>IF(OR(K19="",(E19="Long")*(K19-G19)*J19,(E19="Short")*(G19-K19)*J19))</f>
-        <v/>
-      </c>
-      <c r="N19">
-        <f>IF(G19=0,"",M19/(G19*J19))</f>
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="M19" s="43">
+        <f>IF(OR(E19="",K19=""),"",IF(E19="Long",(K19-G19)*J19,IF(E19="Short",(G19-K19)*J19,"")))</f>
+        <v/>
+      </c>
+      <c r="N19" s="44">
+        <f>IF(OR(E19="",K19="",G19=0),"",IF(E19="Long",(K19-G19)/G19,IF(E19="Short",(G19-K19)/G19,"")))</f>
         <v/>
       </c>
       <c r="O19">
-        <f>IF(OR(G19=H19,J19=0),"",M19/(ABS(G19-H19)*J19))</f>
-        <v/>
-      </c>
-      <c r="Q19">
+        <f>IF(OR(M19="",H19=""),"",IF(ABS(J19*(G19-H19))=0,"N/A",M19/ABS(J19*(G19-H19))))</f>
+        <v/>
+      </c>
+      <c r="Q19" s="43">
         <f>IF(M19="","",M19-P19)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="M20">
-        <f>IF(OR(K20="",(E20="Long")*(K20-G20)*J20,(E20="Short")*(G20-K20)*J20))</f>
-        <v/>
-      </c>
-      <c r="N20">
-        <f>IF(G20=0,"",M20/(G20*J20))</f>
+      <c r="A20" t="n">
+        <v>16</v>
+      </c>
+      <c r="M20" s="43">
+        <f>IF(OR(E20="",K20=""),"",IF(E20="Long",(K20-G20)*J20,IF(E20="Short",(G20-K20)*J20,"")))</f>
+        <v/>
+      </c>
+      <c r="N20" s="44">
+        <f>IF(OR(E20="",K20="",G20=0),"",IF(E20="Long",(K20-G20)/G20,IF(E20="Short",(G20-K20)/G20,"")))</f>
         <v/>
       </c>
       <c r="O20">
-        <f>IF(OR(G20=H20,J20=0),"",M20/(ABS(G20-H20)*J20))</f>
-        <v/>
-      </c>
-      <c r="Q20">
+        <f>IF(OR(M20="",H20=""),"",IF(ABS(J20*(G20-H20))=0,"N/A",M20/ABS(J20*(G20-H20))))</f>
+        <v/>
+      </c>
+      <c r="Q20" s="43">
         <f>IF(M20="","",M20-P20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="M21">
-        <f>IF(OR(K21="",(E21="Long")*(K21-G21)*J21,(E21="Short")*(G21-K21)*J21))</f>
-        <v/>
-      </c>
-      <c r="N21">
-        <f>IF(G21=0,"",M21/(G21*J21))</f>
+      <c r="A21" t="n">
+        <v>17</v>
+      </c>
+      <c r="M21" s="43">
+        <f>IF(OR(E21="",K21=""),"",IF(E21="Long",(K21-G21)*J21,IF(E21="Short",(G21-K21)*J21,"")))</f>
+        <v/>
+      </c>
+      <c r="N21" s="44">
+        <f>IF(OR(E21="",K21="",G21=0),"",IF(E21="Long",(K21-G21)/G21,IF(E21="Short",(G21-K21)/G21,"")))</f>
         <v/>
       </c>
       <c r="O21">
-        <f>IF(OR(G21=H21,J21=0),"",M21/(ABS(G21-H21)*J21))</f>
-        <v/>
-      </c>
-      <c r="Q21">
+        <f>IF(OR(M21="",H21=""),"",IF(ABS(J21*(G21-H21))=0,"N/A",M21/ABS(J21*(G21-H21))))</f>
+        <v/>
+      </c>
+      <c r="Q21" s="43">
         <f>IF(M21="","",M21-P21)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="M22">
-        <f>IF(OR(K22="",(E22="Long")*(K22-G22)*J22,(E22="Short")*(G22-K22)*J22))</f>
-        <v/>
-      </c>
-      <c r="N22">
-        <f>IF(G22=0,"",M22/(G22*J22))</f>
+      <c r="A22" t="n">
+        <v>18</v>
+      </c>
+      <c r="M22" s="43">
+        <f>IF(OR(E22="",K22=""),"",IF(E22="Long",(K22-G22)*J22,IF(E22="Short",(G22-K22)*J22,"")))</f>
+        <v/>
+      </c>
+      <c r="N22" s="44">
+        <f>IF(OR(E22="",K22="",G22=0),"",IF(E22="Long",(K22-G22)/G22,IF(E22="Short",(G22-K22)/G22,"")))</f>
         <v/>
       </c>
       <c r="O22">
-        <f>IF(OR(G22=H22,J22=0),"",M22/(ABS(G22-H22)*J22))</f>
-        <v/>
-      </c>
-      <c r="Q22">
+        <f>IF(OR(M22="",H22=""),"",IF(ABS(J22*(G22-H22))=0,"N/A",M22/ABS(J22*(G22-H22))))</f>
+        <v/>
+      </c>
+      <c r="Q22" s="43">
         <f>IF(M22="","",M22-P22)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="M23">
-        <f>IF(OR(K23="",(E23="Long")*(K23-G23)*J23,(E23="Short")*(G23-K23)*J23))</f>
-        <v/>
-      </c>
-      <c r="N23">
-        <f>IF(G23=0,"",M23/(G23*J23))</f>
+      <c r="A23" t="n">
+        <v>19</v>
+      </c>
+      <c r="M23" s="43">
+        <f>IF(OR(E23="",K23=""),"",IF(E23="Long",(K23-G23)*J23,IF(E23="Short",(G23-K23)*J23,"")))</f>
+        <v/>
+      </c>
+      <c r="N23" s="44">
+        <f>IF(OR(E23="",K23="",G23=0),"",IF(E23="Long",(K23-G23)/G23,IF(E23="Short",(G23-K23)/G23,"")))</f>
         <v/>
       </c>
       <c r="O23">
-        <f>IF(OR(G23=H23,J23=0),"",M23/(ABS(G23-H23)*J23))</f>
-        <v/>
-      </c>
-      <c r="Q23">
+        <f>IF(OR(M23="",H23=""),"",IF(ABS(J23*(G23-H23))=0,"N/A",M23/ABS(J23*(G23-H23))))</f>
+        <v/>
+      </c>
+      <c r="Q23" s="43">
         <f>IF(M23="","",M23-P23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>20</v>
+      </c>
+      <c r="M24" s="43">
+        <f>IF(OR(E24="",K24=""),"",IF(E24="Long",(K24-G24)*J24,IF(E24="Short",(G24-K24)*J24,"")))</f>
+        <v/>
+      </c>
+      <c r="N24" s="44">
+        <f>IF(OR(E24="",K24="",G24=0),"",IF(E24="Long",(K24-G24)/G24,IF(E24="Short",(G24-K24)/G24,"")))</f>
+        <v/>
+      </c>
+      <c r="O24">
+        <f>IF(OR(M24="",H24=""),"",IF(ABS(J24*(G24-H24))=0,"N/A",M24/ABS(J24*(G24-H24))))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="43">
+        <f>IF(M24="","",M24-P24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>21</v>
+      </c>
+      <c r="M25" s="43">
+        <f>IF(OR(E25="",K25=""),"",IF(E25="Long",(K25-G25)*J25,IF(E25="Short",(G25-K25)*J25,"")))</f>
+        <v/>
+      </c>
+      <c r="N25" s="44">
+        <f>IF(OR(E25="",K25="",G25=0),"",IF(E25="Long",(K25-G25)/G25,IF(E25="Short",(G25-K25)/G25,"")))</f>
+        <v/>
+      </c>
+      <c r="O25">
+        <f>IF(OR(M25="",H25=""),"",IF(ABS(J25*(G25-H25))=0,"N/A",M25/ABS(J25*(G25-H25))))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="43">
+        <f>IF(M25="","",M25-P25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>22</v>
+      </c>
+      <c r="M26" s="43">
+        <f>IF(OR(E26="",K26=""),"",IF(E26="Long",(K26-G26)*J26,IF(E26="Short",(G26-K26)*J26,"")))</f>
+        <v/>
+      </c>
+      <c r="N26" s="44">
+        <f>IF(OR(E26="",K26="",G26=0),"",IF(E26="Long",(K26-G26)/G26,IF(E26="Short",(G26-K26)/G26,"")))</f>
+        <v/>
+      </c>
+      <c r="O26">
+        <f>IF(OR(M26="",H26=""),"",IF(ABS(J26*(G26-H26))=0,"N/A",M26/ABS(J26*(G26-H26))))</f>
+        <v/>
+      </c>
+      <c r="Q26" s="43">
+        <f>IF(M26="","",M26-P26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>23</v>
+      </c>
+      <c r="M27" s="43">
+        <f>IF(OR(E27="",K27=""),"",IF(E27="Long",(K27-G27)*J27,IF(E27="Short",(G27-K27)*J27,"")))</f>
+        <v/>
+      </c>
+      <c r="N27" s="44">
+        <f>IF(OR(E27="",K27="",G27=0),"",IF(E27="Long",(K27-G27)/G27,IF(E27="Short",(G27-K27)/G27,"")))</f>
+        <v/>
+      </c>
+      <c r="O27">
+        <f>IF(OR(M27="",H27=""),"",IF(ABS(J27*(G27-H27))=0,"N/A",M27/ABS(J27*(G27-H27))))</f>
+        <v/>
+      </c>
+      <c r="Q27" s="43">
+        <f>IF(M27="","",M27-P27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>24</v>
+      </c>
+      <c r="M28" s="43">
+        <f>IF(OR(E28="",K28=""),"",IF(E28="Long",(K28-G28)*J28,IF(E28="Short",(G28-K28)*J28,"")))</f>
+        <v/>
+      </c>
+      <c r="N28" s="44">
+        <f>IF(OR(E28="",K28="",G28=0),"",IF(E28="Long",(K28-G28)/G28,IF(E28="Short",(G28-K28)/G28,"")))</f>
+        <v/>
+      </c>
+      <c r="O28">
+        <f>IF(OR(M28="",H28=""),"",IF(ABS(J28*(G28-H28))=0,"N/A",M28/ABS(J28*(G28-H28))))</f>
+        <v/>
+      </c>
+      <c r="Q28" s="43">
+        <f>IF(M28="","",M28-P28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>25</v>
+      </c>
+      <c r="M29" s="43">
+        <f>IF(OR(E29="",K29=""),"",IF(E29="Long",(K29-G29)*J29,IF(E29="Short",(G29-K29)*J29,"")))</f>
+        <v/>
+      </c>
+      <c r="N29" s="44">
+        <f>IF(OR(E29="",K29="",G29=0),"",IF(E29="Long",(K29-G29)/G29,IF(E29="Short",(G29-K29)/G29,"")))</f>
+        <v/>
+      </c>
+      <c r="O29">
+        <f>IF(OR(M29="",H29=""),"",IF(ABS(J29*(G29-H29))=0,"N/A",M29/ABS(J29*(G29-H29))))</f>
+        <v/>
+      </c>
+      <c r="Q29" s="43">
+        <f>IF(M29="","",M29-P29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>26</v>
+      </c>
+      <c r="M30" s="43">
+        <f>IF(OR(E30="",K30=""),"",IF(E30="Long",(K30-G30)*J30,IF(E30="Short",(G30-K30)*J30,"")))</f>
+        <v/>
+      </c>
+      <c r="N30" s="44">
+        <f>IF(OR(E30="",K30="",G30=0),"",IF(E30="Long",(K30-G30)/G30,IF(E30="Short",(G30-K30)/G30,"")))</f>
+        <v/>
+      </c>
+      <c r="O30">
+        <f>IF(OR(M30="",H30=""),"",IF(ABS(J30*(G30-H30))=0,"N/A",M30/ABS(J30*(G30-H30))))</f>
+        <v/>
+      </c>
+      <c r="Q30" s="43">
+        <f>IF(M30="","",M30-P30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>27</v>
+      </c>
+      <c r="M31" s="43">
+        <f>IF(OR(E31="",K31=""),"",IF(E31="Long",(K31-G31)*J31,IF(E31="Short",(G31-K31)*J31,"")))</f>
+        <v/>
+      </c>
+      <c r="N31" s="44">
+        <f>IF(OR(E31="",K31="",G31=0),"",IF(E31="Long",(K31-G31)/G31,IF(E31="Short",(G31-K31)/G31,"")))</f>
+        <v/>
+      </c>
+      <c r="O31">
+        <f>IF(OR(M31="",H31=""),"",IF(ABS(J31*(G31-H31))=0,"N/A",M31/ABS(J31*(G31-H31))))</f>
+        <v/>
+      </c>
+      <c r="Q31" s="43">
+        <f>IF(M31="","",M31-P31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>28</v>
+      </c>
+      <c r="M32" s="43">
+        <f>IF(OR(E32="",K32=""),"",IF(E32="Long",(K32-G32)*J32,IF(E32="Short",(G32-K32)*J32,"")))</f>
+        <v/>
+      </c>
+      <c r="N32" s="44">
+        <f>IF(OR(E32="",K32="",G32=0),"",IF(E32="Long",(K32-G32)/G32,IF(E32="Short",(G32-K32)/G32,"")))</f>
+        <v/>
+      </c>
+      <c r="O32">
+        <f>IF(OR(M32="",H32=""),"",IF(ABS(J32*(G32-H32))=0,"N/A",M32/ABS(J32*(G32-H32))))</f>
+        <v/>
+      </c>
+      <c r="Q32" s="43">
+        <f>IF(M32="","",M32-P32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>29</v>
+      </c>
+      <c r="M33" s="43">
+        <f>IF(OR(E33="",K33=""),"",IF(E33="Long",(K33-G33)*J33,IF(E33="Short",(G33-K33)*J33,"")))</f>
+        <v/>
+      </c>
+      <c r="N33" s="44">
+        <f>IF(OR(E33="",K33="",G33=0),"",IF(E33="Long",(K33-G33)/G33,IF(E33="Short",(G33-K33)/G33,"")))</f>
+        <v/>
+      </c>
+      <c r="O33">
+        <f>IF(OR(M33="",H33=""),"",IF(ABS(J33*(G33-H33))=0,"N/A",M33/ABS(J33*(G33-H33))))</f>
+        <v/>
+      </c>
+      <c r="Q33" s="43">
+        <f>IF(M33="","",M33-P33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>30</v>
+      </c>
+      <c r="M34" s="43">
+        <f>IF(OR(E34="",K34=""),"",IF(E34="Long",(K34-G34)*J34,IF(E34="Short",(G34-K34)*J34,"")))</f>
+        <v/>
+      </c>
+      <c r="N34" s="44">
+        <f>IF(OR(E34="",K34="",G34=0),"",IF(E34="Long",(K34-G34)/G34,IF(E34="Short",(G34-K34)/G34,"")))</f>
+        <v/>
+      </c>
+      <c r="O34">
+        <f>IF(OR(M34="",H34=""),"",IF(ABS(J34*(G34-H34))=0,"N/A",M34/ABS(J34*(G34-H34))))</f>
+        <v/>
+      </c>
+      <c r="Q34" s="43">
+        <f>IF(M34="","",M34-P34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>31</v>
+      </c>
+      <c r="M35" s="43">
+        <f>IF(OR(E35="",K35=""),"",IF(E35="Long",(K35-G35)*J35,IF(E35="Short",(G35-K35)*J35,"")))</f>
+        <v/>
+      </c>
+      <c r="N35" s="44">
+        <f>IF(OR(E35="",K35="",G35=0),"",IF(E35="Long",(K35-G35)/G35,IF(E35="Short",(G35-K35)/G35,"")))</f>
+        <v/>
+      </c>
+      <c r="O35">
+        <f>IF(OR(M35="",H35=""),"",IF(ABS(J35*(G35-H35))=0,"N/A",M35/ABS(J35*(G35-H35))))</f>
+        <v/>
+      </c>
+      <c r="Q35" s="43">
+        <f>IF(M35="","",M35-P35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>32</v>
+      </c>
+      <c r="M36" s="43">
+        <f>IF(OR(E36="",K36=""),"",IF(E36="Long",(K36-G36)*J36,IF(E36="Short",(G36-K36)*J36,"")))</f>
+        <v/>
+      </c>
+      <c r="N36" s="44">
+        <f>IF(OR(E36="",K36="",G36=0),"",IF(E36="Long",(K36-G36)/G36,IF(E36="Short",(G36-K36)/G36,"")))</f>
+        <v/>
+      </c>
+      <c r="O36">
+        <f>IF(OR(M36="",H36=""),"",IF(ABS(J36*(G36-H36))=0,"N/A",M36/ABS(J36*(G36-H36))))</f>
+        <v/>
+      </c>
+      <c r="Q36" s="43">
+        <f>IF(M36="","",M36-P36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="M37" s="43">
+        <f>IF(OR(E37="",K37=""),"",IF(E37="Long",(K37-G37)*J37,IF(E37="Short",(G37-K37)*J37,"")))</f>
+        <v/>
+      </c>
+      <c r="N37" s="44">
+        <f>IF(OR(E37="",K37="",G37=0),"",IF(E37="Long",(K37-G37)/G37,IF(E37="Short",(G37-K37)/G37,"")))</f>
+        <v/>
+      </c>
+      <c r="O37">
+        <f>IF(OR(M37="",H37=""),"",IF(ABS(J37*(G37-H37))=0,"N/A",M37/ABS(J37*(G37-H37))))</f>
+        <v/>
+      </c>
+      <c r="Q37" s="43">
+        <f>IF(M37="","",M37-P37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="M38" s="43">
+        <f>IF(OR(E38="",K38=""),"",IF(E38="Long",(K38-G38)*J38,IF(E38="Short",(G38-K38)*J38,"")))</f>
+        <v/>
+      </c>
+      <c r="N38" s="44">
+        <f>IF(OR(E38="",K38="",G38=0),"",IF(E38="Long",(K38-G38)/G38,IF(E38="Short",(G38-K38)/G38,"")))</f>
+        <v/>
+      </c>
+      <c r="O38">
+        <f>IF(OR(M38="",H38=""),"",IF(ABS(J38*(G38-H38))=0,"N/A",M38/ABS(J38*(G38-H38))))</f>
+        <v/>
+      </c>
+      <c r="Q38" s="43">
+        <f>IF(M38="","",M38-P38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="M39" s="43">
+        <f>IF(OR(E39="",K39=""),"",IF(E39="Long",(K39-G39)*J39,IF(E39="Short",(G39-K39)*J39,"")))</f>
+        <v/>
+      </c>
+      <c r="N39" s="44">
+        <f>IF(OR(E39="",K39="",G39=0),"",IF(E39="Long",(K39-G39)/G39,IF(E39="Short",(G39-K39)/G39,"")))</f>
+        <v/>
+      </c>
+      <c r="O39">
+        <f>IF(OR(M39="",H39=""),"",IF(ABS(J39*(G39-H39))=0,"N/A",M39/ABS(J39*(G39-H39))))</f>
+        <v/>
+      </c>
+      <c r="Q39" s="43">
+        <f>IF(M39="","",M39-P39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>36</v>
+      </c>
+      <c r="M40" s="43">
+        <f>IF(OR(E40="",K40=""),"",IF(E40="Long",(K40-G40)*J40,IF(E40="Short",(G40-K40)*J40,"")))</f>
+        <v/>
+      </c>
+      <c r="N40" s="44">
+        <f>IF(OR(E40="",K40="",G40=0),"",IF(E40="Long",(K40-G40)/G40,IF(E40="Short",(G40-K40)/G40,"")))</f>
+        <v/>
+      </c>
+      <c r="O40">
+        <f>IF(OR(M40="",H40=""),"",IF(ABS(J40*(G40-H40))=0,"N/A",M40/ABS(J40*(G40-H40))))</f>
+        <v/>
+      </c>
+      <c r="Q40" s="43">
+        <f>IF(M40="","",M40-P40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>37</v>
+      </c>
+      <c r="M41" s="43">
+        <f>IF(OR(E41="",K41=""),"",IF(E41="Long",(K41-G41)*J41,IF(E41="Short",(G41-K41)*J41,"")))</f>
+        <v/>
+      </c>
+      <c r="N41" s="44">
+        <f>IF(OR(E41="",K41="",G41=0),"",IF(E41="Long",(K41-G41)/G41,IF(E41="Short",(G41-K41)/G41,"")))</f>
+        <v/>
+      </c>
+      <c r="O41">
+        <f>IF(OR(M41="",H41=""),"",IF(ABS(J41*(G41-H41))=0,"N/A",M41/ABS(J41*(G41-H41))))</f>
+        <v/>
+      </c>
+      <c r="Q41" s="43">
+        <f>IF(M41="","",M41-P41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>38</v>
+      </c>
+      <c r="M42" s="43">
+        <f>IF(OR(E42="",K42=""),"",IF(E42="Long",(K42-G42)*J42,IF(E42="Short",(G42-K42)*J42,"")))</f>
+        <v/>
+      </c>
+      <c r="N42" s="44">
+        <f>IF(OR(E42="",K42="",G42=0),"",IF(E42="Long",(K42-G42)/G42,IF(E42="Short",(G42-K42)/G42,"")))</f>
+        <v/>
+      </c>
+      <c r="O42">
+        <f>IF(OR(M42="",H42=""),"",IF(ABS(J42*(G42-H42))=0,"N/A",M42/ABS(J42*(G42-H42))))</f>
+        <v/>
+      </c>
+      <c r="Q42" s="43">
+        <f>IF(M42="","",M42-P42)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>39</v>
+      </c>
+      <c r="M43" s="43">
+        <f>IF(OR(E43="",K43=""),"",IF(E43="Long",(K43-G43)*J43,IF(E43="Short",(G43-K43)*J43,"")))</f>
+        <v/>
+      </c>
+      <c r="N43" s="44">
+        <f>IF(OR(E43="",K43="",G43=0),"",IF(E43="Long",(K43-G43)/G43,IF(E43="Short",(G43-K43)/G43,"")))</f>
+        <v/>
+      </c>
+      <c r="O43">
+        <f>IF(OR(M43="",H43=""),"",IF(ABS(J43*(G43-H43))=0,"N/A",M43/ABS(J43*(G43-H43))))</f>
+        <v/>
+      </c>
+      <c r="Q43" s="43">
+        <f>IF(M43="","",M43-P43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>40</v>
+      </c>
+      <c r="M44" s="43">
+        <f>IF(OR(E44="",K44=""),"",IF(E44="Long",(K44-G44)*J44,IF(E44="Short",(G44-K44)*J44,"")))</f>
+        <v/>
+      </c>
+      <c r="N44" s="44">
+        <f>IF(OR(E44="",K44="",G44=0),"",IF(E44="Long",(K44-G44)/G44,IF(E44="Short",(G44-K44)/G44,"")))</f>
+        <v/>
+      </c>
+      <c r="O44">
+        <f>IF(OR(M44="",H44=""),"",IF(ABS(J44*(G44-H44))=0,"N/A",M44/ABS(J44*(G44-H44))))</f>
+        <v/>
+      </c>
+      <c r="Q44" s="43">
+        <f>IF(M44="","",M44-P44)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>41</v>
+      </c>
+      <c r="M45" s="43">
+        <f>IF(OR(E45="",K45=""),"",IF(E45="Long",(K45-G45)*J45,IF(E45="Short",(G45-K45)*J45,"")))</f>
+        <v/>
+      </c>
+      <c r="N45" s="44">
+        <f>IF(OR(E45="",K45="",G45=0),"",IF(E45="Long",(K45-G45)/G45,IF(E45="Short",(G45-K45)/G45,"")))</f>
+        <v/>
+      </c>
+      <c r="O45">
+        <f>IF(OR(M45="",H45=""),"",IF(ABS(J45*(G45-H45))=0,"N/A",M45/ABS(J45*(G45-H45))))</f>
+        <v/>
+      </c>
+      <c r="Q45" s="43">
+        <f>IF(M45="","",M45-P45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>42</v>
+      </c>
+      <c r="M46" s="43">
+        <f>IF(OR(E46="",K46=""),"",IF(E46="Long",(K46-G46)*J46,IF(E46="Short",(G46-K46)*J46,"")))</f>
+        <v/>
+      </c>
+      <c r="N46" s="44">
+        <f>IF(OR(E46="",K46="",G46=0),"",IF(E46="Long",(K46-G46)/G46,IF(E46="Short",(G46-K46)/G46,"")))</f>
+        <v/>
+      </c>
+      <c r="O46">
+        <f>IF(OR(M46="",H46=""),"",IF(ABS(J46*(G46-H46))=0,"N/A",M46/ABS(J46*(G46-H46))))</f>
+        <v/>
+      </c>
+      <c r="Q46" s="43">
+        <f>IF(M46="","",M46-P46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>43</v>
+      </c>
+      <c r="M47" s="43">
+        <f>IF(OR(E47="",K47=""),"",IF(E47="Long",(K47-G47)*J47,IF(E47="Short",(G47-K47)*J47,"")))</f>
+        <v/>
+      </c>
+      <c r="N47" s="44">
+        <f>IF(OR(E47="",K47="",G47=0),"",IF(E47="Long",(K47-G47)/G47,IF(E47="Short",(G47-K47)/G47,"")))</f>
+        <v/>
+      </c>
+      <c r="O47">
+        <f>IF(OR(M47="",H47=""),"",IF(ABS(J47*(G47-H47))=0,"N/A",M47/ABS(J47*(G47-H47))))</f>
+        <v/>
+      </c>
+      <c r="Q47" s="43">
+        <f>IF(M47="","",M47-P47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>44</v>
+      </c>
+      <c r="M48" s="43">
+        <f>IF(OR(E48="",K48=""),"",IF(E48="Long",(K48-G48)*J48,IF(E48="Short",(G48-K48)*J48,"")))</f>
+        <v/>
+      </c>
+      <c r="N48" s="44">
+        <f>IF(OR(E48="",K48="",G48=0),"",IF(E48="Long",(K48-G48)/G48,IF(E48="Short",(G48-K48)/G48,"")))</f>
+        <v/>
+      </c>
+      <c r="O48">
+        <f>IF(OR(M48="",H48=""),"",IF(ABS(J48*(G48-H48))=0,"N/A",M48/ABS(J48*(G48-H48))))</f>
+        <v/>
+      </c>
+      <c r="Q48" s="43">
+        <f>IF(M48="","",M48-P48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>45</v>
+      </c>
+      <c r="M49" s="43">
+        <f>IF(OR(E49="",K49=""),"",IF(E49="Long",(K49-G49)*J49,IF(E49="Short",(G49-K49)*J49,"")))</f>
+        <v/>
+      </c>
+      <c r="N49" s="44">
+        <f>IF(OR(E49="",K49="",G49=0),"",IF(E49="Long",(K49-G49)/G49,IF(E49="Short",(G49-K49)/G49,"")))</f>
+        <v/>
+      </c>
+      <c r="O49">
+        <f>IF(OR(M49="",H49=""),"",IF(ABS(J49*(G49-H49))=0,"N/A",M49/ABS(J49*(G49-H49))))</f>
+        <v/>
+      </c>
+      <c r="Q49" s="43">
+        <f>IF(M49="","",M49-P49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>46</v>
+      </c>
+      <c r="M50" s="43">
+        <f>IF(OR(E50="",K50=""),"",IF(E50="Long",(K50-G50)*J50,IF(E50="Short",(G50-K50)*J50,"")))</f>
+        <v/>
+      </c>
+      <c r="N50" s="44">
+        <f>IF(OR(E50="",K50="",G50=0),"",IF(E50="Long",(K50-G50)/G50,IF(E50="Short",(G50-K50)/G50,"")))</f>
+        <v/>
+      </c>
+      <c r="O50">
+        <f>IF(OR(M50="",H50=""),"",IF(ABS(J50*(G50-H50))=0,"N/A",M50/ABS(J50*(G50-H50))))</f>
+        <v/>
+      </c>
+      <c r="Q50" s="43">
+        <f>IF(M50="","",M50-P50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>47</v>
+      </c>
+      <c r="M51" s="43">
+        <f>IF(OR(E51="",K51=""),"",IF(E51="Long",(K51-G51)*J51,IF(E51="Short",(G51-K51)*J51,"")))</f>
+        <v/>
+      </c>
+      <c r="N51" s="44">
+        <f>IF(OR(E51="",K51="",G51=0),"",IF(E51="Long",(K51-G51)/G51,IF(E51="Short",(G51-K51)/G51,"")))</f>
+        <v/>
+      </c>
+      <c r="O51">
+        <f>IF(OR(M51="",H51=""),"",IF(ABS(J51*(G51-H51))=0,"N/A",M51/ABS(J51*(G51-H51))))</f>
+        <v/>
+      </c>
+      <c r="Q51" s="43">
+        <f>IF(M51="","",M51-P51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>48</v>
+      </c>
+      <c r="M52" s="43">
+        <f>IF(OR(E52="",K52=""),"",IF(E52="Long",(K52-G52)*J52,IF(E52="Short",(G52-K52)*J52,"")))</f>
+        <v/>
+      </c>
+      <c r="N52" s="44">
+        <f>IF(OR(E52="",K52="",G52=0),"",IF(E52="Long",(K52-G52)/G52,IF(E52="Short",(G52-K52)/G52,"")))</f>
+        <v/>
+      </c>
+      <c r="O52">
+        <f>IF(OR(M52="",H52=""),"",IF(ABS(J52*(G52-H52))=0,"N/A",M52/ABS(J52*(G52-H52))))</f>
+        <v/>
+      </c>
+      <c r="Q52" s="43">
+        <f>IF(M52="","",M52-P52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>49</v>
+      </c>
+      <c r="M53" s="43">
+        <f>IF(OR(E53="",K53=""),"",IF(E53="Long",(K53-G53)*J53,IF(E53="Short",(G53-K53)*J53,"")))</f>
+        <v/>
+      </c>
+      <c r="N53" s="44">
+        <f>IF(OR(E53="",K53="",G53=0),"",IF(E53="Long",(K53-G53)/G53,IF(E53="Short",(G53-K53)/G53,"")))</f>
+        <v/>
+      </c>
+      <c r="O53">
+        <f>IF(OR(M53="",H53=""),"",IF(ABS(J53*(G53-H53))=0,"N/A",M53/ABS(J53*(G53-H53))))</f>
+        <v/>
+      </c>
+      <c r="Q53" s="43">
+        <f>IF(M53="","",M53-P53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>50</v>
+      </c>
+      <c r="M54" s="43">
+        <f>IF(OR(E54="",K54=""),"",IF(E54="Long",(K54-G54)*J54,IF(E54="Short",(G54-K54)*J54,"")))</f>
+        <v/>
+      </c>
+      <c r="N54" s="44">
+        <f>IF(OR(E54="",K54="",G54=0),"",IF(E54="Long",(K54-G54)/G54,IF(E54="Short",(G54-K54)/G54,"")))</f>
+        <v/>
+      </c>
+      <c r="O54">
+        <f>IF(OR(M54="",H54=""),"",IF(ABS(J54*(G54-H54))=0,"N/A",M54/ABS(J54*(G54-H54))))</f>
+        <v/>
+      </c>
+      <c r="Q54" s="43">
+        <f>IF(M54="","",M54-P54)</f>
         <v/>
       </c>
     </row>
@@ -1330,11 +2108,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>TRADING DASHBOARD</t>
         </is>
       </c>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1450,16 +2231,15 @@
         </is>
       </c>
       <c r="B9" s="22">
-        <f>IF(COUNTIF('📋 Trade Log'!M5:M1000,"&gt;0")=0,0,MAX('📋 Trade Log'!M5:M1000))</f>
-        <v/>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>WORST TRADE</t>
-        </is>
+        <f>COUNTA('📋 Trade Log'!E5:E1000)</f>
+        <v/>
+      </c>
+      <c r="C9" s="19">
+        <f>IF(B9=0,"0%",COUNTIF('📋 Trade Log'!Q5:Q1000,"&gt;0")/B9)</f>
+        <v/>
       </c>
       <c r="D9" s="22">
-        <f>IF(COUNTIF('📋 Trade Log'!M5:M1000,"&lt;0")=0,0,MIN('📋 Trade Log'!M5:M1000))</f>
+        <f>SUM('📋 Trade Log'!Q5:Q1000)</f>
         <v/>
       </c>
     </row>
@@ -1470,33 +2250,34 @@
         </is>
       </c>
       <c r="B10" s="24">
-        <f>IF(COUNTA('📋 Trade Log'!L5:L1000)=0,"N/A",AVERAGE('📋 Trade Log'!L5:L1000-'📋 Trade Log'!B5:B1000))</f>
-        <v/>
-      </c>
-      <c r="C10" s="19" t="inlineStr">
-        <is>
-          <t>COMMISSION TOTAL</t>
-        </is>
+        <f>IF(COUNTA('📋 Trade Log'!L5:L1000)=0,"N/A",SUMPRODUCT(('📋 Trade Log'!L5:L1000-'📋 Trade Log'!B5:B1000)*('📋 Trade Log'!L5:L1000&lt;&gt;""))/COUNTA('📋 Trade Log'!L5:L1000))</f>
+        <v/>
+      </c>
+      <c r="C10" s="19">
+        <f>IF(COUNTIF('📋 Trade Log'!Q5:Q1000,"&gt;0")=0,"N/A",AVERAGEIF('📋 Trade Log'!Q5:Q1000,"&gt;0"))</f>
+        <v/>
       </c>
       <c r="D10" s="22">
-        <f>SUM('📋 Trade Log'!P5:P1000)</f>
+        <f>IF(COUNTIF('📋 Trade Log'!Q5:Q1000,"&lt;0")=0,"N/A",AVERAGEIF('📋 Trade Log'!Q5:Q1000,"&lt;0"))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>CURRENT STREAK</t>
-        </is>
-      </c>
-      <c r="B11" s="20" t="inlineStr"/>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>MAX DRAWDOWN</t>
-        </is>
+          <t>WORST TRADE</t>
+        </is>
+      </c>
+      <c r="B11" s="20">
+        <f>IF(COUNTA('📋 Trade Log'!Q5:Q1000)=0,"",INDEX('📋 Trade Log'!Q5:Q1000,COUNTA('📋 Trade Log'!Q5:Q1000)))</f>
+        <v/>
+      </c>
+      <c r="C11" s="19">
+        <f>IF(SUMIF('📋 Trade Log'!Q5:Q1000,"&gt;0")=0,"N/A",SUMIF('📋 Trade Log'!Q5:Q1000,"&gt;0")/ABS(SUMIF('📋 Trade Log'!Q5:Q1000,"&lt;0")))</f>
+        <v/>
       </c>
       <c r="D11" s="22">
-        <f>MIN('📋 Trade Log'!M5:M1000)</f>
+        <f>IF(COUNTA('📋 Trade Log'!Q5:Q1000)=0,"",MIN('📋 Trade Log'!Q5:Q1000))</f>
         <v/>
       </c>
     </row>
@@ -1809,7 +2590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1824,11 +2605,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>TRADING ANALYTICS</t>
         </is>
       </c>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -2103,10 +2887,8 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
-        <is>
-          <t>MONTHLY PERFORMANCE</t>
-        </is>
+      <c r="A14" s="25" t="n">
+        <v>9</v>
       </c>
       <c r="B14" s="5">
         <f>INDEX('📋 Trade Log'!B5:B1000,9)</f>
@@ -2122,360 +2904,362 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>Trades</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>Win Rate</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>Gross P&amp;L</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>Net P&amp;L</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Avg R</t>
-        </is>
-      </c>
+      <c r="A15" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" s="32">
+        <f>INDEX('📋 Trade Log'!B5:B1000,10)</f>
+        <v/>
+      </c>
+      <c r="C15" s="33">
+        <f>INDEX('📋 Trade Log'!Q5:Q1000,10)</f>
+        <v/>
+      </c>
+      <c r="D15" s="33">
+        <f>D14+C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="45" t="inlineStr">
+        <is>
+          <t>MONTHLY PERFORMANCE</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="34" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="35" t="n"/>
+      <c r="F16" s="36" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="50" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="B16" s="5">
+      <c r="B17" s="51">
         <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01")</f>
         <v/>
       </c>
-      <c r="C16" s="34">
-        <f>IF(B16=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B16)</f>
-        <v/>
-      </c>
-      <c r="D16" s="6">
+      <c r="C17" s="52">
+        <f>IF(B17=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01")/B17)</f>
+        <v/>
+      </c>
+      <c r="D17" s="53">
         <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01")</f>
         <v/>
       </c>
-      <c r="E16" s="35">
+      <c r="E17" s="54">
         <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01")</f>
         <v/>
       </c>
-      <c r="F16" s="36">
-        <f>IF(B16=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Feb</t>
-        </is>
-      </c>
-      <c r="B17" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")</f>
-        <v/>
-      </c>
-      <c r="C17" s="34">
-        <f>IF(B17=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B17)</f>
-        <v/>
-      </c>
-      <c r="D17" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")</f>
-        <v/>
-      </c>
-      <c r="E17" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")</f>
-        <v/>
-      </c>
-      <c r="F17" s="36">
-        <f>IF(B17=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01"))</f>
+      <c r="F17" s="55">
+        <f>IF(B17=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-01-01",'📋 Trade Log'!B5:B1000,"&lt;2026-02-01"))</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Feb</t>
         </is>
       </c>
       <c r="B18" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")</f>
         <v/>
       </c>
       <c r="C18" s="34">
-        <f>IF(B18=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B18)</f>
+        <f>IF(B18=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")/B18)</f>
         <v/>
       </c>
       <c r="D18" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")</f>
         <v/>
       </c>
       <c r="E18" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01")</f>
         <v/>
       </c>
       <c r="F18" s="36">
-        <f>IF(B18=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01"))</f>
+        <f>IF(B18=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-02-01",'📋 Trade Log'!B5:B1000,"&lt;2026-03-01"))</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Apr</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="B19" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")</f>
         <v/>
       </c>
       <c r="C19" s="34">
-        <f>IF(B19=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B19)</f>
+        <f>IF(B19=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")/B19)</f>
         <v/>
       </c>
       <c r="D19" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")</f>
         <v/>
       </c>
       <c r="E19" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01")</f>
         <v/>
       </c>
       <c r="F19" s="36">
-        <f>IF(B19=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01"))</f>
+        <f>IF(B19=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-03-01",'📋 Trade Log'!B5:B1000,"&lt;2026-04-01"))</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>May</t>
+          <t>Apr</t>
         </is>
       </c>
       <c r="B20" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")</f>
         <v/>
       </c>
       <c r="C20" s="34">
-        <f>IF(B20=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B20)</f>
+        <f>IF(B20=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")/B20)</f>
         <v/>
       </c>
       <c r="D20" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")</f>
         <v/>
       </c>
       <c r="E20" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01")</f>
         <v/>
       </c>
       <c r="F20" s="36">
-        <f>IF(B20=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01"))</f>
+        <f>IF(B20=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-04-01",'📋 Trade Log'!B5:B1000,"&lt;2026-05-01"))</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Jun</t>
+          <t>May</t>
         </is>
       </c>
       <c r="B21" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")</f>
         <v/>
       </c>
       <c r="C21" s="34">
-        <f>IF(B21=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B21)</f>
+        <f>IF(B21=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")/B21)</f>
         <v/>
       </c>
       <c r="D21" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")</f>
         <v/>
       </c>
       <c r="E21" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01")</f>
         <v/>
       </c>
       <c r="F21" s="36">
-        <f>IF(B21=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01"))</f>
+        <f>IF(B21=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-05-01",'📋 Trade Log'!B5:B1000,"&lt;2026-06-01"))</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Jul</t>
+          <t>Jun</t>
         </is>
       </c>
       <c r="B22" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")</f>
         <v/>
       </c>
       <c r="C22" s="34">
-        <f>IF(B22=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B22)</f>
+        <f>IF(B22=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")/B22)</f>
         <v/>
       </c>
       <c r="D22" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")</f>
         <v/>
       </c>
       <c r="E22" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01")</f>
         <v/>
       </c>
       <c r="F22" s="36">
-        <f>IF(B22=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01"))</f>
+        <f>IF(B22=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-06-01",'📋 Trade Log'!B5:B1000,"&lt;2026-07-01"))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Aug</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="B23" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")</f>
         <v/>
       </c>
       <c r="C23" s="34">
-        <f>IF(B23=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B23)</f>
+        <f>IF(B23=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")/B23)</f>
         <v/>
       </c>
       <c r="D23" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")</f>
         <v/>
       </c>
       <c r="E23" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01")</f>
         <v/>
       </c>
       <c r="F23" s="36">
-        <f>IF(B23=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01"))</f>
+        <f>IF(B23=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-07-01",'📋 Trade Log'!B5:B1000,"&lt;2026-08-01"))</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Sep</t>
+          <t>Aug</t>
         </is>
       </c>
       <c r="B24" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")</f>
         <v/>
       </c>
       <c r="C24" s="34">
-        <f>IF(B24=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B24)</f>
+        <f>IF(B24=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")/B24)</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")</f>
         <v/>
       </c>
       <c r="E24" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01")</f>
         <v/>
       </c>
       <c r="F24" s="36">
-        <f>IF(B24=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01"))</f>
+        <f>IF(B24=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-08-01",'📋 Trade Log'!B5:B1000,"&lt;2026-09-01"))</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Oct</t>
+          <t>Sep</t>
         </is>
       </c>
       <c r="B25" s="5">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")</f>
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")</f>
         <v/>
       </c>
       <c r="C25" s="34">
-        <f>IF(B25=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B25)</f>
+        <f>IF(B25=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")/B25)</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")</f>
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")</f>
         <v/>
       </c>
       <c r="E25" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01")</f>
         <v/>
       </c>
       <c r="F25" s="36">
-        <f>IF(B25=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01"))</f>
+        <f>IF(B25=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-09-01",'📋 Trade Log'!B5:B1000,"&lt;2026-10-01"))</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Nov</t>
-        </is>
-      </c>
-      <c r="B26" s="30">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")</f>
-        <v/>
-      </c>
-      <c r="C26" s="31">
-        <f>IF(B26=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B26)</f>
-        <v/>
-      </c>
-      <c r="D26" s="35">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")</f>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B26" s="4">
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")</f>
+        <v/>
+      </c>
+      <c r="C26" s="34">
+        <f>IF(B26=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")/B26)</f>
+        <v/>
+      </c>
+      <c r="D26" s="6">
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")</f>
         <v/>
       </c>
       <c r="E26" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")</f>
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01")</f>
         <v/>
       </c>
       <c r="F26" s="36">
-        <f>IF(B26=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01"))</f>
+        <f>IF(B26=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-10-01",'📋 Trade Log'!B5:B1000,"&lt;2026-11-01"))</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B27" s="30">
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")</f>
+        <v/>
+      </c>
+      <c r="C27" s="31">
+        <f>IF(B27=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")/B27)</f>
+        <v/>
+      </c>
+      <c r="D27" s="35">
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")</f>
+        <v/>
+      </c>
+      <c r="E27" s="35">
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01")</f>
+        <v/>
+      </c>
+      <c r="F27" s="36">
+        <f>IF(B27=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-11-01",'📋 Trade Log'!B5:B1000,"&lt;2026-12-01"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="48" t="inlineStr">
+        <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="B27" s="30">
-        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2026-13-01")</f>
-        <v/>
-      </c>
-      <c r="C27" s="31">
-        <f>IF(B27=0,"N/A",COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2026-13-01",'📋 Trade Log'!M5:M1000,"&gt;0")/B27)</f>
-        <v/>
-      </c>
-      <c r="D27" s="35">
-        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2026-13-01")</f>
-        <v/>
-      </c>
-      <c r="E27" s="35">
-        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2026-13-01")</f>
-        <v/>
-      </c>
-      <c r="F27" s="36">
-        <f>IF(B27=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2026-13-01"))</f>
-        <v/>
-      </c>
+      <c r="B28">
+        <f>COUNTIFS('📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2027-01-01")</f>
+        <v/>
+      </c>
+      <c r="C28">
+        <f>IF(B28=0,"N/A",COUNTIFS('📋 Trade Log'!Q5:Q1000,"&gt;0",'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2027-01-01")/B28)</f>
+        <v/>
+      </c>
+      <c r="D28">
+        <f>SUMIFS('📋 Trade Log'!M5:M1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2027-01-01")</f>
+        <v/>
+      </c>
+      <c r="E28">
+        <f>SUMIFS('📋 Trade Log'!Q5:Q1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2027-01-01")</f>
+        <v/>
+      </c>
+      <c r="F28">
+        <f>IF(B28=0,"N/A",AVERAGEIFS('📋 Trade Log'!O5:O1000,'📋 Trade Log'!B5:B1000,"&gt;=2026-12-01",'📋 Trade Log'!B5:B1000,"&lt;2027-01-01"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2500,11 +3284,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="49" t="inlineStr">
         <is>
           <t>PRO TRADING JOURNAL</t>
         </is>
       </c>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">

</xml_diff>